<commit_message>
feat: align capacity analysis pages with excel prototypes
</commit_message>
<xml_diff>
--- a/aps-system/src/main/resources/static/template-bom.xlsx
+++ b/aps-system/src/main/resources/static/template-bom.xlsx
@@ -2,41 +2,210 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="14055" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="25">
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <i val="1"/>
-      <color rgb="007F6000"/>
+      <color rgb="FF7F6000"/>
       <sz val="10"/>
-    </font>
-    <font>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="35">
     <fill>
       <patternFill/>
     </fill>
@@ -45,16 +214,204 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001B4F8A"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B4F8A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -64,23 +421,266 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -88,10 +688,72 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -444,7 +1106,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -454,24 +1115,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:M13"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="7" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>说明：按版本号进行全删全导；无子零件行为叶节点工艺行；报废率范围[0,1)；版本号必填</t>
         </is>
@@ -505,64 +1163,642 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>模腔数/取数(pcs)</t>
+          <t>制造部门</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>制造周期(S)</t>
+          <t>制造单元</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>持台人数(人)</t>
+          <t>模腔数/取数（pcs）</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>单件节拍(S)</t>
+          <t>制造周期（S）</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
+          <t>持台人数（人）</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>单件节拍（S）</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
           <t>报废率</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>版本号</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n"/>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>11201A012</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>11201A012-1</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>aa</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>aa001</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>制造一部</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>单元A</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>20260331-1</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>11201A012-1</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>21201A012</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>bb</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>bb001</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>制造一部</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>单元A</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>20260331-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>11201A012-1</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>11201A012-1-1</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>bb</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>bb001</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>制造一部</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>单元A</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>20260331-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>11201A012-1-1</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>31201A012</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>cc</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>cc001</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>制造二部</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>单元B</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>20260331-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>11201A012-1-1</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>31201A013</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>cc</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>cc001</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>制造二部</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>单元B</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>20260331-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>21201A012</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>31201A014</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>dd</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>dd001</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>制造二部</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>单元C</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>20260331-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>31201A013</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>41201A012</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>ee</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>ee001</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>制造三部</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>单元D</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>20260331-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>41201A012</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>ff</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>ff001</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>制造三部</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>单元D</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>20260331-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>11201A022</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>21201A022</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>aa</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>aa001</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>制造一部</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>单元A</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>20260331-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>21201A022</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>31201A022</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>bb</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>bb002</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>制造二部</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>单元E</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>20260331-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>31201A022</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>cc</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>cc002</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>制造二部</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>单元E</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>20260331-1</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: sync APS workspace to GitLab
</commit_message>
<xml_diff>
--- a/aps-system/src/main/resources/static/template-bom.xlsx
+++ b/aps-system/src/main/resources/static/template-bom.xlsx
@@ -18,7 +18,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="22">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -44,13 +44,6 @@
     </font>
     <font>
       <name val="宋体"/>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
       <charset val="0"/>
       <color rgb="FF0000FF"/>
       <sz val="11"/>
@@ -192,17 +185,6 @@
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="35">
@@ -534,174 +516,168 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1115,690 +1091,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="17.125" customWidth="1" min="1" max="2"/>
+    <col width="5.375" customWidth="1" min="3" max="4"/>
+    <col width="8.375" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="9.375" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="7.375" customWidth="1" min="12" max="12"/>
+    <col width="13.75" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>说明：按版本号进行全删全导；无子零件行为叶节点工艺行；报废率范围[0,1)；版本号必填</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>根完成品</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>父零件</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>子零件</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>用量</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>工序</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>设备</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>制造部门</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>制造单元</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>模腔数/取数（pcs）</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>制造周期（S）</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>持台人数（人）</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>单件节拍（S）</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>报废率</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>版本号</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>11201A012</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>11201A012-1</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>aa</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>aa001</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>制造一部</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>单元A</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="J3" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="L3" s="6" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="M3" s="6" t="inlineStr">
-        <is>
-          <t>20260331-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>11201A012-1</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>21201A012</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>bb</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>bb001</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>制造一部</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>单元A</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="J4" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="L4" s="6" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="M4" s="6" t="inlineStr">
-        <is>
-          <t>20260331-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>11201A012-1</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>11201A012-1-1</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>bb</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>bb001</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>制造一部</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>单元A</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>20260331-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>11201A012-1-1</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>31201A012</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>cc</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>cc001</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>制造二部</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>单元B</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="L6" s="6" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="M6" s="6" t="inlineStr">
-        <is>
-          <t>20260331-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>11201A012-1-1</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>31201A013</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>cc</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>cc001</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>制造二部</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>单元B</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="M7" s="6" t="inlineStr">
-        <is>
-          <t>20260331-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>21201A012</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>31201A014</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>dd</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>dd001</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>制造二部</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>单元C</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="J8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="L8" s="6" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="M8" s="6" t="inlineStr">
-        <is>
-          <t>20260331-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>31201A013</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>41201A012</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>ee</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>ee001</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>制造三部</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>单元D</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="M9" s="6" t="inlineStr">
-        <is>
-          <t>20260331-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>41201A012</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>ff</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>ff001</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>制造三部</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>单元D</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" s="6" t="n">
-        <v>37</v>
-      </c>
-      <c r="J10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="6" t="n">
-        <v>37</v>
-      </c>
-      <c r="L10" s="6" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="M10" s="6" t="inlineStr">
-        <is>
-          <t>20260331-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>11201A022</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>21201A022</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>aa</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>aa001</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>制造一部</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>单元A</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="J11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="M11" s="6" t="inlineStr">
-        <is>
-          <t>20260331-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>21201A022</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>31201A022</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>bb</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>bb002</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>制造二部</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>单元E</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="J12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="L12" s="6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="M12" s="6" t="inlineStr">
-        <is>
-          <t>20260331-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>31201A022</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>cc</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>cc002</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>制造二部</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>单元E</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="J13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="L13" s="6" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="M13" s="6" t="inlineStr">
-        <is>
-          <t>20260331-1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A1:M1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix APS BOM and capacity calculation rules
</commit_message>
<xml_diff>
--- a/aps-system/src/main/resources/static/template-bom.xlsx
+++ b/aps-system/src/main/resources/static/template-bom.xlsx
@@ -1091,7 +1091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="17.125" customWidth="1" min="1" max="2"/>
@@ -1182,13 +1182,18 @@
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
+          <t>子零件属性</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
           <t>版本号</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>